<commit_message>
Add zoom controls and functionality to the app
</commit_message>
<xml_diff>
--- a/Danh_sach_playlist_Da_Co_Anh.xlsx
+++ b/Danh_sach_playlist_Da_Co_Anh.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\pjsk\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\pjsk\event-collection\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9B34007-DFCC-443D-A8F6-41452DFEB9DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED667A23-3E57-4BE2-A2B9-E689CC687D1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="57">
   <si>
     <t>STT</t>
   </si>
@@ -188,13 +188,16 @@
   </si>
   <si>
     <t>https://res.cloudinary.com/logocollection/image/upload/v1774513652/event_sekai/event_188.jpg</t>
+  </si>
+  <si>
+    <t>Toàn lực! Wonder Halloween!</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -207,6 +210,18 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -216,7 +231,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -239,14 +254,38 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -550,7 +589,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -592,7 +631,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -606,197 +645,195 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" t="s">
-        <v>14</v>
+    <row r="4" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="C7" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D7" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C8" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D8" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C9" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D9" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C10" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D10" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>74</v>
+        <v>29</v>
       </c>
       <c r="B11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C11" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D11" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C12" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D12" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="B13" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D13" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="B14" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C14" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D14" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="B15" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C15" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D15" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>145</v>
+        <v>111</v>
       </c>
       <c r="B16" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C16" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D16" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="B17" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C17" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D17" t="s">
         <v>11</v>
@@ -804,13 +841,13 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>170</v>
+        <v>150</v>
       </c>
       <c r="B18" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C18" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D18" t="s">
         <v>11</v>
@@ -818,13 +855,13 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="B19" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C19" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D19" t="s">
         <v>11</v>
@@ -832,57 +869,71 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="B20" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C20" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D20" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B21" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C21" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D21" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B22" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C22" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D22" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23">
+        <v>185</v>
+      </c>
+      <c r="B23" t="s">
+        <v>52</v>
+      </c>
+      <c r="C23" t="s">
+        <v>53</v>
+      </c>
+      <c r="D23" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24">
         <v>188</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B24" t="s">
         <v>54</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C24" t="s">
         <v>55</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D24" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>